<commit_message>
fix: resolve missing positions during employee imports
</commit_message>
<xml_diff>
--- a/resources/templates/plantilla-importacion-funcionarios-sigal.xlsx
+++ b/resources/templates/plantilla-importacion-funcionarios-sigal.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Funcionarios" sheetId="1" r:id="R47e856bdb8f64dcf"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Guia de llenado" sheetId="2" r:id="R3d7796ff6ec64b18"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Funcionarios" sheetId="1" r:id="R4cbbfe6d25f84f26"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Guia de llenado" sheetId="2" r:id="R60aa8f162abc4248"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -11075,7 +11075,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4ecc5232acc64547"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd9bf44ec7d5249d2"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -11196,7 +11196,7 @@
     </x:row>
     <x:row r="6" ht="31" customHeight="1">
       <x:c r="A6" s="27" t="str">
-        <x:v>En codigo_oficina elija el nombre completo de la oficina. El cargo debe coincidir exactamente con un cargo vigente de esa oficina en SIGAL.</x:v>
+        <x:v>En codigo_oficina elija el nombre completo de la oficina. Si el cargo no existe, SIGAL solicitará clasificarlo como Funcionario o Responsable antes de importar.</x:v>
       </x:c>
       <x:c r="B6" s="27"/>
       <x:c r="C6" s="27"/>

</xml_diff>